<commit_message>
fix: 标注表 xlsx 被 Excel/WPS 拒载——列分组缺 outlineLevelCol 声明
- 根因：OOXML 要求列带 outlineLevel 时 sheet 级须声明 outlineLevelCol；
  openpyxl group() 不自动补，且保存器用 column_dimensions.max_outline(初始None)
  覆盖 sheet_format 手动值——正确挂点是 ws.column_dimensions.max_outline=1
- 颜色改全 8 位 ARGB(FF 前缀)：openpyxl 对 6 位值补 00-alpha，WPS 渲染成透明
- 回归测试锚住两点（readback 断言 outlineLevelCol==1 + FFFFF2CC）
- 以往错误.md 增 §6 记录该坑（openpyxl 读回验证不算数，要拆 zip 看 XML）

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/annotation/标注表模板.xlsx
+++ b/data/annotation/标注表模板.xlsx
@@ -27,7 +27,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <color rgb="00808080"/>
+      <color rgb="FF808080"/>
     </font>
     <font>
       <b val="1"/>
@@ -35,7 +35,7 @@
     <font/>
     <font>
       <i val="1"/>
-      <color rgb="00808080"/>
+      <color rgb="FF808080"/>
     </font>
   </fonts>
   <fills count="5">
@@ -47,17 +47,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E7E6E6"/>
+        <fgColor rgb="FFE7E6E6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DDEBF7"/>
+        <fgColor rgb="FFDDEBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -445,7 +445,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AM4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="1"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col hidden="1" outlineLevel="1" width="14" customWidth="1" min="2" max="4"/>

</xml_diff>